<commit_message>
Limpa status das transacoes de exemplo para permitir novo teste
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Automacao_Correios/input/transacoes.xlsx
+++ b/Automacao_Correios/input/transacoes.xlsx
@@ -30,9 +30,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">NN437873753BR </x:t>
-  </x:si>
-  <x:si>
-    <x:t>ok</x:t>
   </x:si>
   <x:si>
     <x:t>AP612167199BR</x:t>
@@ -370,15 +367,9 @@
       <x:c r="A2" s="2" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
     </x:row>
     <x:row r="3" spans="1:3">
       <x:c r="A3" s="2" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
         <x:v>3</x:v>
       </x:c>
     </x:row>

</xml_diff>